<commit_message>
gih data 2025 processed added headings original data
</commit_message>
<xml_diff>
--- a/data/gih/original_data/gih-2025.xlsx
+++ b/data/gih/original_data/gih-2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\APC-fond\Open APC Sweden\Tidigare inskickat till KB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2021m30/R/repos/openapc-se/data/gih/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B965B0-5F4F-4A3E-8BAC-223B0F7E445F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAD8502-2A08-8D43-855D-E4EFFEDCF47E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{62BBDB78-9CB0-4DCF-ADD9-9A13FB04FC4C}"/>
+    <workbookView xWindow="90480" yWindow="7860" windowWidth="19420" windowHeight="11500" xr2:uid="{62BBDB78-9CB0-4DCF-ADD9-9A13FB04FC4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="35">
   <si>
     <t>gih</t>
   </si>
@@ -108,6 +108,39 @@
   </si>
   <si>
     <t>0888-4781</t>
+  </si>
+  <si>
+    <t>institution</t>
+  </si>
+  <si>
+    <t>period</t>
+  </si>
+  <si>
+    <t>sek</t>
+  </si>
+  <si>
+    <t>doi</t>
+  </si>
+  <si>
+    <t>is_hybrid</t>
+  </si>
+  <si>
+    <t>publisher</t>
+  </si>
+  <si>
+    <t>journal_full_title</t>
+  </si>
+  <si>
+    <t>issn</t>
+  </si>
+  <si>
+    <t>issn_print</t>
+  </si>
+  <si>
+    <t>issn_electronic</t>
+  </si>
+  <si>
+    <t>url</t>
   </si>
 </sst>
 </file>
@@ -525,36 +558,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0799543-F1FE-447F-8A44-AC6DB25BC15F}">
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="44.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1">
-        <v>2025</v>
-      </c>
-      <c r="C1" s="8">
-        <v>35194</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>9</v>
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>29</v>
       </c>
       <c r="G1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -562,77 +607,77 @@
         <v>2025</v>
       </c>
       <c r="C2" s="8">
-        <v>38465</v>
+        <v>35194</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>20</v>
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3">
         <v>2025</v>
       </c>
-      <c r="C3" s="3">
-        <v>16893.55</v>
+      <c r="C3" s="8">
+        <v>38465</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>21</v>
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4">
         <v>2025</v>
       </c>
-      <c r="C4" s="8">
-        <v>1874</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>4</v>
+      <c r="C4" s="3">
+        <v>16893.55</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>22</v>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -640,25 +685,25 @@
         <v>2025</v>
       </c>
       <c r="C5" s="8">
-        <v>32801</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>5</v>
+        <v>1874</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>23</v>
+        <v>17</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -666,10 +711,10 @@
         <v>2025</v>
       </c>
       <c r="C6" s="8">
-        <v>28497.82</v>
+        <v>32801</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" t="s">
         <v>8</v>
@@ -681,6 +726,32 @@
         <v>18</v>
       </c>
       <c r="H6" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7">
+        <v>2025</v>
+      </c>
+      <c r="C7" s="8">
+        <v>28497.82</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>23</v>
       </c>
     </row>

</xml_diff>